<commit_message>
Updated backend with new Aiven DB connection
</commit_message>
<xml_diff>
--- a/attendance/yearly_exl_file/2026/March_2026.xlsx
+++ b/attendance/yearly_exl_file/2026/March_2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>ID</t>
   </si>
@@ -25,27 +25,6 @@
     <t>Domain</t>
   </si>
   <si>
-    <t>11/3/2026 [Wed]</t>
-  </si>
-  <si>
-    <t>12/3/2026 [Thu]</t>
-  </si>
-  <si>
-    <t>13/3/2026 [Fri]</t>
-  </si>
-  <si>
-    <t>14/3/2026 [Sat]</t>
-  </si>
-  <si>
-    <t>15/3/2026 [Sun]</t>
-  </si>
-  <si>
-    <t>16/3/2026 [Mon]</t>
-  </si>
-  <si>
-    <t>17/3/2026 [Tue]</t>
-  </si>
-  <si>
     <t>18/3/2026 [Wed]</t>
   </si>
   <si>
@@ -115,6 +94,27 @@
     <t>9/4/2026 [Thu]</t>
   </si>
   <si>
+    <t>10/4/2026 [Fri]</t>
+  </si>
+  <si>
+    <t>11/4/2026 [Sat]</t>
+  </si>
+  <si>
+    <t>12/4/2026 [Sun]</t>
+  </si>
+  <si>
+    <t>13/4/2026 [Mon]</t>
+  </si>
+  <si>
+    <t>14/4/2026 [Tue]</t>
+  </si>
+  <si>
+    <t>15/4/2026 [Wed]</t>
+  </si>
+  <si>
+    <t>16/4/2026 [Thu]</t>
+  </si>
+  <si>
     <t>DNYANESHWAR SHARAD TIDME</t>
   </si>
   <si>
@@ -122,15 +122,6 @@
   </si>
   <si>
     <t>Full Stack MERN</t>
-  </si>
-  <si>
-    <t>P</t>
-  </si>
-  <si>
-    <t xml:space="preserve">yogesh surywanshi </t>
-  </si>
-  <si>
-    <t>Data Analytics</t>
   </si>
 </sst>
 </file>
@@ -174,11 +165,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -518,7 +508,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AH3"/>
+  <dimension ref="A1:AH2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -631,9 +621,9 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>756700</v>
+        <v>466448</v>
       </c>
       <c r="B2" t="s">
         <v>34</v>
@@ -643,42 +633,10 @@
       </c>
       <c r="D2" t="s">
         <v>36</v>
-      </c>
-      <c r="E2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F2" t="s">
-        <v>37</v>
-      </c>
-      <c r="G2" t="s">
-        <v>37</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="J2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>222076</v>
-      </c>
-      <c r="B3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D3" t="s">
-        <v>39</v>
-      </c>
-      <c r="G3" t="s">
-        <v>37</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated backend use gps location mark
</commit_message>
<xml_diff>
--- a/attendance/yearly_exl_file/2026/March_2026.xlsx
+++ b/attendance/yearly_exl_file/2026/March_2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="39">
   <si>
     <t>ID</t>
   </si>
@@ -122,6 +122,12 @@
   </si>
   <si>
     <t>Full Stack MERN</t>
+  </si>
+  <si>
+    <t>Data Analytics</t>
+  </si>
+  <si>
+    <t>P</t>
   </si>
 </sst>
 </file>
@@ -508,7 +514,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AH2"/>
+  <dimension ref="A1:AH3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -635,8 +641,25 @@
         <v>36</v>
       </c>
     </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>190068</v>
+      </c>
+      <c r="B3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E3" t="s">
+        <v>38</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>